<commit_message>
Complete Stage 2 inventory model and documentation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Inventory_Model.xlsx
+++ b/data/Inventory_Model.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,21 +11,34 @@
     <sheet name="Results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Mu">Inputs!$B$2</definedName>
-    <definedName name="Sigma">Inputs!$B$3</definedName>
+    <definedName name="AnnualDemand">Results!$B$2</definedName>
     <definedName name="DaysPerYear">Inputs!$B$4</definedName>
-    <definedName name="OrderCost">Inputs!$B$5</definedName>
+    <definedName name="EOQ_Q">Results!$B$3</definedName>
     <definedName name="HoldCost">Inputs!$B$6</definedName>
     <definedName name="LeadTime">Inputs!$B$7</definedName>
+    <definedName name="Mu">Inputs!$B$2</definedName>
+    <definedName name="OrderCost">Inputs!$B$5</definedName>
+    <definedName name="ReorderPoint">Results!$B$8</definedName>
+    <definedName name="SafetyStock">Results!$B$7</definedName>
     <definedName name="ServiceLevel">Inputs!$B$8</definedName>
+    <definedName name="Sigma">Inputs!$B$3</definedName>
+    <definedName name="TotalCost">Results!$B$12</definedName>
     <definedName name="z_value">Inputs!$B$9</definedName>
-    <definedName name="AnnualDemand">Results!$B$2</definedName>
-    <definedName name="EOQ_Q">Results!$B$3</definedName>
-    <definedName name="SafetyStock">Results!$B$7</definedName>
-    <definedName name="ReorderPoint">Results!$B$8</definedName>
-    <definedName name="TotalCost">Results!$B$12</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -115,9 +127,11 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0"/>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -192,11 +206,13 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <roundedCorners val="0"/>
+  <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
           <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -228,6 +244,7 @@
       </spPr>
     </title>
     <plotArea>
+      <layout/>
       <lineChart>
         <grouping val="standard"/>
         <varyColors val="0"/>
@@ -244,7 +261,6 @@
           </spPr>
           <marker>
             <symbol val="none"/>
-            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -253,12 +269,200 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Demand'!$A$2:$A$31</f>
+              <f>Demand!$A$2:$A$31</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="30"/>
+                <pt idx="0">
+                  <v>1</v>
+                </pt>
+                <pt idx="1">
+                  <v>2</v>
+                </pt>
+                <pt idx="2">
+                  <v>3</v>
+                </pt>
+                <pt idx="3">
+                  <v>4</v>
+                </pt>
+                <pt idx="4">
+                  <v>5</v>
+                </pt>
+                <pt idx="5">
+                  <v>6</v>
+                </pt>
+                <pt idx="6">
+                  <v>7</v>
+                </pt>
+                <pt idx="7">
+                  <v>8</v>
+                </pt>
+                <pt idx="8">
+                  <v>9</v>
+                </pt>
+                <pt idx="9">
+                  <v>10</v>
+                </pt>
+                <pt idx="10">
+                  <v>11</v>
+                </pt>
+                <pt idx="11">
+                  <v>12</v>
+                </pt>
+                <pt idx="12">
+                  <v>13</v>
+                </pt>
+                <pt idx="13">
+                  <v>14</v>
+                </pt>
+                <pt idx="14">
+                  <v>15</v>
+                </pt>
+                <pt idx="15">
+                  <v>16</v>
+                </pt>
+                <pt idx="16">
+                  <v>17</v>
+                </pt>
+                <pt idx="17">
+                  <v>18</v>
+                </pt>
+                <pt idx="18">
+                  <v>19</v>
+                </pt>
+                <pt idx="19">
+                  <v>20</v>
+                </pt>
+                <pt idx="20">
+                  <v>21</v>
+                </pt>
+                <pt idx="21">
+                  <v>22</v>
+                </pt>
+                <pt idx="22">
+                  <v>23</v>
+                </pt>
+                <pt idx="23">
+                  <v>24</v>
+                </pt>
+                <pt idx="24">
+                  <v>25</v>
+                </pt>
+                <pt idx="25">
+                  <v>26</v>
+                </pt>
+                <pt idx="26">
+                  <v>27</v>
+                </pt>
+                <pt idx="27">
+                  <v>28</v>
+                </pt>
+                <pt idx="28">
+                  <v>29</v>
+                </pt>
+                <pt idx="29">
+                  <v>30</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Demand'!$C$2:$C$31</f>
+              <f>Demand!$C$2:$C$31</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="30"/>
+                <pt idx="0">
+                  <v>40</v>
+                </pt>
+                <pt idx="1">
+                  <v>53</v>
+                </pt>
+                <pt idx="2">
+                  <v>27</v>
+                </pt>
+                <pt idx="3">
+                  <v>67</v>
+                </pt>
+                <pt idx="4">
+                  <v>58</v>
+                </pt>
+                <pt idx="5">
+                  <v>46</v>
+                </pt>
+                <pt idx="6">
+                  <v>46</v>
+                </pt>
+                <pt idx="7">
+                  <v>54</v>
+                </pt>
+                <pt idx="8">
+                  <v>47</v>
+                </pt>
+                <pt idx="9">
+                  <v>47</v>
+                </pt>
+                <pt idx="10">
+                  <v>59</v>
+                </pt>
+                <pt idx="11">
+                  <v>56</v>
+                </pt>
+                <pt idx="12">
+                  <v>49</v>
+                </pt>
+                <pt idx="13">
+                  <v>49</v>
+                </pt>
+                <pt idx="14">
+                  <v>52</v>
+                </pt>
+                <pt idx="15">
+                  <v>42</v>
+                </pt>
+                <pt idx="16">
+                  <v>45</v>
+                </pt>
+                <pt idx="17">
+                  <v>57</v>
+                </pt>
+                <pt idx="18">
+                  <v>48</v>
+                </pt>
+                <pt idx="19">
+                  <v>33</v>
+                </pt>
+                <pt idx="20">
+                  <v>44</v>
+                </pt>
+                <pt idx="21">
+                  <v>58</v>
+                </pt>
+                <pt idx="22">
+                  <v>47</v>
+                </pt>
+                <pt idx="23">
+                  <v>48</v>
+                </pt>
+                <pt idx="24">
+                  <v>58</v>
+                </pt>
+                <pt idx="25">
+                  <v>73</v>
+                </pt>
+                <pt idx="26">
+                  <v>41</v>
+                </pt>
+                <pt idx="27">
+                  <v>67</v>
+                </pt>
+                <pt idx="28">
+                  <v>35</v>
+                </pt>
+                <pt idx="29">
+                  <v>52</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -276,7 +480,6 @@
           </spPr>
           <marker>
             <symbol val="none"/>
-            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -285,17 +488,213 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Demand'!$A$2:$A$31</f>
+              <f>Demand!$A$2:$A$31</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="30"/>
+                <pt idx="0">
+                  <v>1</v>
+                </pt>
+                <pt idx="1">
+                  <v>2</v>
+                </pt>
+                <pt idx="2">
+                  <v>3</v>
+                </pt>
+                <pt idx="3">
+                  <v>4</v>
+                </pt>
+                <pt idx="4">
+                  <v>5</v>
+                </pt>
+                <pt idx="5">
+                  <v>6</v>
+                </pt>
+                <pt idx="6">
+                  <v>7</v>
+                </pt>
+                <pt idx="7">
+                  <v>8</v>
+                </pt>
+                <pt idx="8">
+                  <v>9</v>
+                </pt>
+                <pt idx="9">
+                  <v>10</v>
+                </pt>
+                <pt idx="10">
+                  <v>11</v>
+                </pt>
+                <pt idx="11">
+                  <v>12</v>
+                </pt>
+                <pt idx="12">
+                  <v>13</v>
+                </pt>
+                <pt idx="13">
+                  <v>14</v>
+                </pt>
+                <pt idx="14">
+                  <v>15</v>
+                </pt>
+                <pt idx="15">
+                  <v>16</v>
+                </pt>
+                <pt idx="16">
+                  <v>17</v>
+                </pt>
+                <pt idx="17">
+                  <v>18</v>
+                </pt>
+                <pt idx="18">
+                  <v>19</v>
+                </pt>
+                <pt idx="19">
+                  <v>20</v>
+                </pt>
+                <pt idx="20">
+                  <v>21</v>
+                </pt>
+                <pt idx="21">
+                  <v>22</v>
+                </pt>
+                <pt idx="22">
+                  <v>23</v>
+                </pt>
+                <pt idx="23">
+                  <v>24</v>
+                </pt>
+                <pt idx="24">
+                  <v>25</v>
+                </pt>
+                <pt idx="25">
+                  <v>26</v>
+                </pt>
+                <pt idx="26">
+                  <v>27</v>
+                </pt>
+                <pt idx="27">
+                  <v>28</v>
+                </pt>
+                <pt idx="28">
+                  <v>29</v>
+                </pt>
+                <pt idx="29">
+                  <v>30</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Demand'!$D$2:$D$31</f>
+              <f>Demand!$D$2:$D$31</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="30"/>
+                <pt idx="0">
+                  <v>50</v>
+                </pt>
+                <pt idx="1">
+                  <v>50</v>
+                </pt>
+                <pt idx="2">
+                  <v>50</v>
+                </pt>
+                <pt idx="3">
+                  <v>50</v>
+                </pt>
+                <pt idx="4">
+                  <v>50</v>
+                </pt>
+                <pt idx="5">
+                  <v>50</v>
+                </pt>
+                <pt idx="6">
+                  <v>50</v>
+                </pt>
+                <pt idx="7">
+                  <v>50</v>
+                </pt>
+                <pt idx="8">
+                  <v>50</v>
+                </pt>
+                <pt idx="9">
+                  <v>50</v>
+                </pt>
+                <pt idx="10">
+                  <v>50</v>
+                </pt>
+                <pt idx="11">
+                  <v>50</v>
+                </pt>
+                <pt idx="12">
+                  <v>50</v>
+                </pt>
+                <pt idx="13">
+                  <v>50</v>
+                </pt>
+                <pt idx="14">
+                  <v>50</v>
+                </pt>
+                <pt idx="15">
+                  <v>50</v>
+                </pt>
+                <pt idx="16">
+                  <v>50</v>
+                </pt>
+                <pt idx="17">
+                  <v>50</v>
+                </pt>
+                <pt idx="18">
+                  <v>50</v>
+                </pt>
+                <pt idx="19">
+                  <v>50</v>
+                </pt>
+                <pt idx="20">
+                  <v>50</v>
+                </pt>
+                <pt idx="21">
+                  <v>50</v>
+                </pt>
+                <pt idx="22">
+                  <v>50</v>
+                </pt>
+                <pt idx="23">
+                  <v>50</v>
+                </pt>
+                <pt idx="24">
+                  <v>50</v>
+                </pt>
+                <pt idx="25">
+                  <v>50</v>
+                </pt>
+                <pt idx="26">
+                  <v>50</v>
+                </pt>
+                <pt idx="27">
+                  <v>50</v>
+                </pt>
+                <pt idx="28">
+                  <v>50</v>
+                </pt>
+                <pt idx="29">
+                  <v>50</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
           <smooth val="0"/>
         </ser>
-        <marker val="1"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <smooth val="0"/>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -310,6 +709,7 @@
           <tx>
             <rich>
               <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -359,6 +759,7 @@
         </spPr>
         <txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -408,6 +809,7 @@
           <tx>
             <rich>
               <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -451,6 +853,7 @@
         </spPr>
         <txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -492,6 +895,7 @@
       </spPr>
       <txPr>
         <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -534,11 +938,13 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <roundedCorners val="0"/>
+  <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
           <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -570,6 +976,7 @@
       </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -587,16 +994,49 @@
           </spPr>
           <invertIfNegative val="0"/>
           <cat>
-            <numRef>
-              <f>'Results'!$A$6:$A$8</f>
-            </numRef>
+            <strRef>
+              <f>Results!$A$6:$A$8</f>
+              <strCache>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>Lead-time demand</v>
+                </pt>
+                <pt idx="1">
+                  <v>Safety stock (SS)</v>
+                </pt>
+                <pt idx="2">
+                  <v>Reorder point (ROP)</v>
+                </pt>
+              </strCache>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Results'!$B$6:$B$8</f>
+              <f>Results!$B$6:$B$8</f>
+              <numCache>
+                <formatCode>0.0</formatCode>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>250</v>
+                </pt>
+                <pt idx="1">
+                  <v>36.78004522900571</v>
+                </pt>
+                <pt idx="2">
+                  <v>286.7800452290057</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
         <gapWidth val="219"/>
         <overlap val="-27"/>
         <axId val="10"/>
@@ -628,6 +1068,7 @@
         </spPr>
         <txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -677,6 +1118,7 @@
           <tx>
             <rich>
               <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -707,7 +1149,7 @@
             </a:ln>
           </spPr>
         </title>
-        <numFmt formatCode="General" sourceLinked="1"/>
+        <numFmt formatCode="0.0" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
@@ -720,6 +1162,7 @@
         </spPr>
         <txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
@@ -1114,7 +1557,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1245,7 +1688,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>NORMSINV(B8)</f>
+        <f>_xlfn.NORM.S.INV(B8)</f>
         <v/>
       </c>
     </row>
@@ -1261,7 +1704,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
@@ -1827,7 +2270,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>

</xml_diff>